<commit_message>
deploy: Appium E2E Report – Build #4 (d050f83aeb1788eb551414de208f9ebd9553b0c3) d050f83aeb1788eb551414de208f9ebd9553b0c3
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.1</v>
+        <v>0.241</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.1</v>
+        <v>0.241</v>
       </c>
     </row>
     <row r="3">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>20.45</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05 03:28:45 UTC</t>
+          <t>2026-08-05 03:51:30 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #5 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.241</v>
+        <v>0.25</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.241</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="3">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>20.46</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05 03:51:30 UTC</t>
+          <t>2026-08-05 04:09:35 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #6 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.25</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.25</v>
+        <v>0.08799999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="22">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.46</t>
+          <t>20.28</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05 04:09:35 UTC</t>
+          <t>2026-08-05 05:18:43 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #7 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.216</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.216</v>
       </c>
     </row>
     <row r="3">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="6">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="22">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.28</t>
+          <t>20.44</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05 05:18:43 UTC</t>
+          <t>2026-08-06 05:20:10 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #8 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.216</v>
+        <v>0.274</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
     </row>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="F462" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G462" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.216</v>
+        <v>0.274</v>
       </c>
     </row>
     <row r="3">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="11">
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="42">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -19134,7 +19134,7 @@
         </is>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -19734,7 +19734,7 @@
         </is>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="203">
@@ -24234,7 +24234,7 @@
         </is>
       </c>
       <c r="F262" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="284">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="364">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="387">
@@ -30234,7 +30234,7 @@
         </is>
       </c>
       <c r="F462" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="463">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.44</t>
+          <t>20.43</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-06 05:20:10 UTC</t>
+          <t>2026-08-07 04:30:29 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #9 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.274</v>
+        <v>0.21</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
     </row>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
     </row>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="F462" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G462" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.274</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="3">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="11">
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="13">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="42">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -19134,7 +19134,7 @@
         </is>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="93">
@@ -19734,7 +19734,7 @@
         </is>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="113">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="143">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="144">
@@ -24234,7 +24234,7 @@
         </is>
       </c>
       <c r="F262" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="263">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -30234,7 +30234,7 @@
         </is>
       </c>
       <c r="F462" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="463">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.43</t>
+          <t>20.39</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-07 04:30:29 UTC</t>
+          <t>2026-08-08 03:29:10 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #10 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.21</v>
+        <v>0.362</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14923,7 +14923,7 @@
         </is>
       </c>
       <c r="F465" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G465" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.21</v>
+        <v>0.362</v>
       </c>
     </row>
     <row r="3">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="23">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="33">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="42">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="267">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="284">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="364">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="387">
@@ -30324,7 +30324,7 @@
         </is>
       </c>
       <c r="F465" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="466">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.39</t>
+          <t>20.54</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-08 03:29:10 UTC</t>
+          <t>2026-08-09 03:44:59 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #11 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.362</v>
+        <v>0.275</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8072,7 +8072,7 @@
         </is>
       </c>
       <c r="F244" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -14923,7 +14923,7 @@
         </is>
       </c>
       <c r="F465" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G465" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.362</v>
+        <v>0.275</v>
       </c>
     </row>
     <row r="3">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="10">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="23">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="33">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="42">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="144">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="203">
@@ -23694,7 +23694,7 @@
         </is>
       </c>
       <c r="F244" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="245">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="267">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -30324,7 +30324,7 @@
         </is>
       </c>
       <c r="F465" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="466">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.54</t>
+          <t>20.50</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-09 03:44:59 UTC</t>
+          <t>2026-08-10 03:56:45 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #12 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.275</v>
+        <v>0.163</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8072,7 +8072,7 @@
         </is>
       </c>
       <c r="F244" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.275</v>
+        <v>0.163</v>
       </c>
     </row>
     <row r="3">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="203">
@@ -23694,7 +23694,7 @@
         </is>
       </c>
       <c r="F244" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="245">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.50</t>
+          <t>20.36</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-10 03:56:45 UTC</t>
+          <t>2026-08-11 03:46:41 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #13 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.163</v>
+        <v>0.1</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.163</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="96">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.36</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-11 03:46:41 UTC</t>
+          <t>2026-08-12 04:10:36 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #14 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.1</v>
+        <v>0.246</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="F243" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G243" s="2" t="inlineStr"/>
     </row>
@@ -8072,7 +8072,7 @@
         </is>
       </c>
       <c r="F244" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.1</v>
+        <v>0.246</v>
       </c>
     </row>
     <row r="3">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="11">
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="30">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -23664,7 +23664,7 @@
         </is>
       </c>
       <c r="F243" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="244">
@@ -23694,7 +23694,7 @@
         </is>
       </c>
       <c r="F244" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="245">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="364">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>20.46</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-12 04:10:36 UTC</t>
+          <t>2026-08-13 04:16:24 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #15 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.246</v>
+        <v>0.141</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.246</v>
+        <v>0.141</v>
       </c>
     </row>
     <row r="3">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.46</t>
+          <t>20.36</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-13 04:16:24 UTC</t>
+          <t>2026-08-14 04:11:54 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #16 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.141</v>
+        <v>0.514</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.141</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="3">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.36</t>
+          <t>20.72</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-14 04:11:54 UTC</t>
+          <t>2026-08-15 02:55:04 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #17 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.514</v>
+        <v>0.202</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
     </row>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
     </row>
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G113" s="2" t="inlineStr"/>
     </row>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
     </row>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G115" s="2" t="inlineStr"/>
     </row>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
     </row>
@@ -4135,7 +4135,7 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G117" s="2" t="inlineStr"/>
     </row>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -4972,7 +4972,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
     </row>
@@ -5530,7 +5530,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G162" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5592,7 +5592,7 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G164" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="F243" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G243" s="2" t="inlineStr"/>
     </row>
@@ -8072,7 +8072,7 @@
         </is>
       </c>
       <c r="F244" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
     </row>
@@ -8103,7 +8103,7 @@
         </is>
       </c>
       <c r="F245" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G245" s="2" t="inlineStr"/>
     </row>
@@ -8134,7 +8134,7 @@
         </is>
       </c>
       <c r="F246" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G246" s="2" t="inlineStr"/>
     </row>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
     </row>
@@ -8661,7 +8661,7 @@
         </is>
       </c>
       <c r="F263" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G263" s="2" t="inlineStr"/>
     </row>
@@ -8692,7 +8692,7 @@
         </is>
       </c>
       <c r="F264" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G264" s="2" t="inlineStr"/>
     </row>
@@ -8723,7 +8723,7 @@
         </is>
       </c>
       <c r="F265" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G265" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="F362" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G362" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -11792,7 +11792,7 @@
         </is>
       </c>
       <c r="F364" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G364" s="2" t="inlineStr"/>
     </row>
@@ -12350,7 +12350,7 @@
         </is>
       </c>
       <c r="F382" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G382" s="2" t="inlineStr"/>
     </row>
@@ -12381,7 +12381,7 @@
         </is>
       </c>
       <c r="F383" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G383" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14272,7 +14272,7 @@
         </is>
       </c>
       <c r="F444" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G444" s="2" t="inlineStr"/>
     </row>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="F462" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G462" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14892,7 +14892,7 @@
         </is>
       </c>
       <c r="F464" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G464" s="2" t="inlineStr"/>
     </row>
@@ -14923,7 +14923,7 @@
         </is>
       </c>
       <c r="F465" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G465" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -14985,7 +14985,7 @@
         </is>
       </c>
       <c r="F467" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G467" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.514</v>
+        <v>0.202</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="11">
@@ -16704,7 +16704,7 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="42">
@@ -17634,7 +17634,7 @@
         </is>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -18534,7 +18534,7 @@
         </is>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -19134,7 +19134,7 @@
         </is>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -19734,7 +19734,7 @@
         </is>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -19764,7 +19764,7 @@
         </is>
       </c>
       <c r="F113" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -19794,7 +19794,7 @@
         </is>
       </c>
       <c r="F114" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115">
@@ -19824,7 +19824,7 @@
         </is>
       </c>
       <c r="F115" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -19854,7 +19854,7 @@
         </is>
       </c>
       <c r="F116" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -19884,7 +19884,7 @@
         </is>
       </c>
       <c r="F117" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -20694,7 +20694,7 @@
         </is>
       </c>
       <c r="F144" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -21234,7 +21234,7 @@
         </is>
       </c>
       <c r="F162" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="164">
@@ -21294,7 +21294,7 @@
         </is>
       </c>
       <c r="F164" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="203">
@@ -23664,7 +23664,7 @@
         </is>
       </c>
       <c r="F243" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="244">
@@ -23694,7 +23694,7 @@
         </is>
       </c>
       <c r="F244" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245">
@@ -23724,7 +23724,7 @@
         </is>
       </c>
       <c r="F245" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246">
@@ -23754,7 +23754,7 @@
         </is>
       </c>
       <c r="F246" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247">
@@ -24234,7 +24234,7 @@
         </is>
       </c>
       <c r="F262" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263">
@@ -24264,7 +24264,7 @@
         </is>
       </c>
       <c r="F263" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="264">
@@ -24294,7 +24294,7 @@
         </is>
       </c>
       <c r="F264" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265">
@@ -24324,7 +24324,7 @@
         </is>
       </c>
       <c r="F265" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="266">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="284">
@@ -27234,7 +27234,7 @@
         </is>
       </c>
       <c r="F362" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
@@ -27294,7 +27294,7 @@
         </is>
       </c>
       <c r="F364" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365">
@@ -27834,7 +27834,7 @@
         </is>
       </c>
       <c r="F382" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="383">
@@ -27864,7 +27864,7 @@
         </is>
       </c>
       <c r="F383" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="384">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="387">
@@ -29694,7 +29694,7 @@
         </is>
       </c>
       <c r="F444" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="445">
@@ -30234,7 +30234,7 @@
         </is>
       </c>
       <c r="F462" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="463">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="464">
@@ -30294,7 +30294,7 @@
         </is>
       </c>
       <c r="F464" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="465">
@@ -30324,7 +30324,7 @@
         </is>
       </c>
       <c r="F465" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="466">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -30384,7 +30384,7 @@
         </is>
       </c>
       <c r="F467" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="468">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.72</t>
+          <t>20.33</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15 02:55:04 UTC</t>
+          <t>2026-08-16 03:03:53 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #18 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.202</v>
+        <v>0.331</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
     </row>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
     </row>
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G113" s="2" t="inlineStr"/>
     </row>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
     </row>
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G115" s="2" t="inlineStr"/>
     </row>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
     </row>
@@ -4135,7 +4135,7 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G117" s="2" t="inlineStr"/>
     </row>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -4972,7 +4972,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5530,7 +5530,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G162" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5592,7 +5592,7 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G164" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="F243" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G243" s="2" t="inlineStr"/>
     </row>
@@ -8072,7 +8072,7 @@
         </is>
       </c>
       <c r="F244" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
     </row>
@@ -8103,7 +8103,7 @@
         </is>
       </c>
       <c r="F245" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G245" s="2" t="inlineStr"/>
     </row>
@@ -8134,7 +8134,7 @@
         </is>
       </c>
       <c r="F246" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G246" s="2" t="inlineStr"/>
     </row>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
     </row>
@@ -8661,7 +8661,7 @@
         </is>
       </c>
       <c r="F263" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G263" s="2" t="inlineStr"/>
     </row>
@@ -8692,7 +8692,7 @@
         </is>
       </c>
       <c r="F264" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G264" s="2" t="inlineStr"/>
     </row>
@@ -8723,7 +8723,7 @@
         </is>
       </c>
       <c r="F265" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G265" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="F362" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G362" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -11792,7 +11792,7 @@
         </is>
       </c>
       <c r="F364" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G364" s="2" t="inlineStr"/>
     </row>
@@ -12350,7 +12350,7 @@
         </is>
       </c>
       <c r="F382" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G382" s="2" t="inlineStr"/>
     </row>
@@ -12381,7 +12381,7 @@
         </is>
       </c>
       <c r="F383" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G383" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14272,7 +14272,7 @@
         </is>
       </c>
       <c r="F444" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G444" s="2" t="inlineStr"/>
     </row>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="F462" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G462" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14892,7 +14892,7 @@
         </is>
       </c>
       <c r="F464" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G464" s="2" t="inlineStr"/>
     </row>
@@ -14923,7 +14923,7 @@
         </is>
       </c>
       <c r="F465" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G465" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -14985,7 +14985,7 @@
         </is>
       </c>
       <c r="F467" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G467" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.202</v>
+        <v>0.331</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="11">
@@ -16704,7 +16704,7 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="12">
@@ -16734,7 +16734,7 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="42">
@@ -17634,7 +17634,7 @@
         </is>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="43">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -18534,7 +18534,7 @@
         </is>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="73">
@@ -19134,7 +19134,7 @@
         </is>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="93">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -19734,7 +19734,7 @@
         </is>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="113">
@@ -19764,7 +19764,7 @@
         </is>
       </c>
       <c r="F113" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="114">
@@ -19794,7 +19794,7 @@
         </is>
       </c>
       <c r="F114" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="115">
@@ -19824,7 +19824,7 @@
         </is>
       </c>
       <c r="F115" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="116">
@@ -19854,7 +19854,7 @@
         </is>
       </c>
       <c r="F116" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="117">
@@ -19884,7 +19884,7 @@
         </is>
       </c>
       <c r="F117" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="118">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="143">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="144">
@@ -20694,7 +20694,7 @@
         </is>
       </c>
       <c r="F144" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="145">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -21234,7 +21234,7 @@
         </is>
       </c>
       <c r="F162" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="163">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="164">
@@ -21294,7 +21294,7 @@
         </is>
       </c>
       <c r="F164" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="165">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="203">
@@ -23664,7 +23664,7 @@
         </is>
       </c>
       <c r="F243" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="244">
@@ -23694,7 +23694,7 @@
         </is>
       </c>
       <c r="F244" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="245">
@@ -23724,7 +23724,7 @@
         </is>
       </c>
       <c r="F245" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="246">
@@ -23754,7 +23754,7 @@
         </is>
       </c>
       <c r="F246" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="247">
@@ -24234,7 +24234,7 @@
         </is>
       </c>
       <c r="F262" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="263">
@@ -24264,7 +24264,7 @@
         </is>
       </c>
       <c r="F263" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="264">
@@ -24294,7 +24294,7 @@
         </is>
       </c>
       <c r="F264" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="265">
@@ -24324,7 +24324,7 @@
         </is>
       </c>
       <c r="F265" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="266">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -27234,7 +27234,7 @@
         </is>
       </c>
       <c r="F362" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="363">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="364">
@@ -27294,7 +27294,7 @@
         </is>
       </c>
       <c r="F364" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="365">
@@ -27834,7 +27834,7 @@
         </is>
       </c>
       <c r="F382" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="383">
@@ -27864,7 +27864,7 @@
         </is>
       </c>
       <c r="F383" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="384">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="387">
@@ -29694,7 +29694,7 @@
         </is>
       </c>
       <c r="F444" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="445">
@@ -30234,7 +30234,7 @@
         </is>
       </c>
       <c r="F462" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="463">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="464">
@@ -30294,7 +30294,7 @@
         </is>
       </c>
       <c r="F464" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="465">
@@ -30324,7 +30324,7 @@
         </is>
       </c>
       <c r="F465" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="466">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="467">
@@ -30384,7 +30384,7 @@
         </is>
       </c>
       <c r="F467" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="468">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.33</t>
+          <t>20.54</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-16 03:03:53 UTC</t>
+          <t>2026-08-17 03:02:42 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #19 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.331</v>
+        <v>0.195</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.331</v>
+        <v>0.195</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="11">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="22">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="33">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="203">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="284">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="387">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.54</t>
+          <t>21.10</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-17 03:02:42 UTC</t>
+          <t>2026-08-18 02:59:38 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #20 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.195</v>
+        <v>0.099</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.195</v>
+        <v>0.099</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="11">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="22">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="29">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="33">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="38">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="203">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="387">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>21.10</t>
+          <t>20.31</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-18 02:59:38 UTC</t>
+          <t>2026-08-19 03:00:56 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #21 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.099</v>
+        <v>0.258</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
     </row>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5530,7 +5530,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G162" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="F462" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G462" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.099</v>
+        <v>0.258</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="11">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="42">
@@ -17634,7 +17634,7 @@
         </is>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -18534,7 +18534,7 @@
         </is>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -19134,7 +19134,7 @@
         </is>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -19734,7 +19734,7 @@
         </is>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -21234,7 +21234,7 @@
         </is>
       </c>
       <c r="F162" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="203">
@@ -24234,7 +24234,7 @@
         </is>
       </c>
       <c r="F262" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="284">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="387">
@@ -30234,7 +30234,7 @@
         </is>
       </c>
       <c r="F462" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="463">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.31</t>
+          <t>20.40</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-19 03:00:56 UTC</t>
+          <t>2026-08-20 03:00:00 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #22 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.258</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
     </row>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
     </row>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -5530,7 +5530,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G162" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8630,7 +8630,7 @@
         </is>
       </c>
       <c r="F262" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G282" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="F462" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G462" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.258</v>
+        <v>0.08699999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="11">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="14">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="42">
@@ -17634,7 +17634,7 @@
         </is>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="43">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="45">
@@ -18534,7 +18534,7 @@
         </is>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="73">
@@ -19134,7 +19134,7 @@
         </is>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="93">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -19734,7 +19734,7 @@
         </is>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="113">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="143">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="144">
@@ -21234,7 +21234,7 @@
         </is>
       </c>
       <c r="F162" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="163">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="203">
@@ -24234,7 +24234,7 @@
         </is>
       </c>
       <c r="F262" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="263">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="267">
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="F282" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="283">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="364">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="387">
@@ -30234,7 +30234,7 @@
         </is>
       </c>
       <c r="F462" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="463">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.40</t>
+          <t>20.28</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-20 03:00:00 UTC</t>
+          <t>2026-08-21 03:05:36 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #23 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.164</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.164</v>
       </c>
     </row>
     <row r="3">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="7">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.28</t>
+          <t>20.38</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-21 03:05:36 UTC</t>
+          <t>2026-08-22 02:57:31 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #24 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.164</v>
+        <v>0.243</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.164</v>
+        <v>0.243</v>
       </c>
     </row>
     <row r="3">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.38</t>
+          <t>20.46</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-22 02:57:31 UTC</t>
+          <t>2026-08-23 03:05:03 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #25 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.243</v>
+        <v>0.106</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.243</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="3">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.46</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23 03:05:03 UTC</t>
+          <t>2026-08-24 03:05:46 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #26 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.106</v>
+        <v>0.221</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.106</v>
+        <v>0.221</v>
       </c>
     </row>
     <row r="3">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="166">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>20.42</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-24 03:05:46 UTC</t>
+          <t>2026-08-25 03:01:14 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #27 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.221</v>
+        <v>0.091</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.221</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="3">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="166">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.42</t>
+          <t>20.29</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-25 03:01:14 UTC</t>
+          <t>2026-08-26 03:07:50 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #28 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.091</v>
+        <v>0.233</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.091</v>
+        <v>0.233</v>
       </c>
     </row>
     <row r="3">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.29</t>
+          <t>20.45</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-26 03:07:50 UTC</t>
+          <t>2026-08-27 12:26:46 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #29 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.233</v>
+        <v>0.171</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.233</v>
+        <v>0.171</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="11">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="42">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="203">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="267">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="284">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="387">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-27 12:26:46 UTC</t>
+          <t>2026-08-28 13:51:56 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #30 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.171</v>
+        <v>0.158</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
     </row>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
     </row>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -4941,7 +4941,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G165" s="2" t="inlineStr"/>
     </row>
@@ -6770,7 +6770,7 @@
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
     </row>
@@ -8754,7 +8754,7 @@
         </is>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G266" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="F283" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G283" s="2" t="inlineStr"/>
     </row>
@@ -11761,7 +11761,7 @@
         </is>
       </c>
       <c r="F363" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G363" s="2" t="inlineStr"/>
     </row>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F386" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G386" s="2" t="inlineStr"/>
     </row>
@@ -14861,7 +14861,7 @@
         </is>
       </c>
       <c r="F463" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G463" s="2" t="inlineStr"/>
     </row>
@@ -14954,7 +14954,7 @@
         </is>
       </c>
       <c r="F466" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G466" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.171</v>
+        <v>0.158</v>
       </c>
     </row>
     <row r="3">
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">
@@ -16524,7 +16524,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -16554,7 +16554,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="7">
@@ -16584,7 +16584,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -16644,7 +16644,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="10">
@@ -16674,7 +16674,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="11">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="14">
@@ -16794,7 +16794,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="15">
@@ -16824,7 +16824,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="16">
@@ -16854,7 +16854,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -16974,7 +16974,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="21">
@@ -17004,7 +17004,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="22">
@@ -17034,7 +17034,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="23">
@@ -17064,7 +17064,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="24">
@@ -17094,7 +17094,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -17124,7 +17124,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="26">
@@ -17154,7 +17154,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="27">
@@ -17184,7 +17184,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="28">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="30">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="31">
@@ -17304,7 +17304,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="33">
@@ -17364,7 +17364,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="34">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="36">
@@ -17454,7 +17454,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="37">
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="38">
@@ -17514,7 +17514,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="39">
@@ -17544,7 +17544,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="40">
@@ -17574,7 +17574,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="41">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="42">
@@ -17694,7 +17694,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="45">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19224,7 +19224,7 @@
         </is>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="96">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -20664,7 +20664,7 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="144">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="164">
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="166">
@@ -22434,7 +22434,7 @@
         </is>
       </c>
       <c r="F202" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="203">
@@ -24354,7 +24354,7 @@
         </is>
       </c>
       <c r="F266" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="267">
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="F363" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="364">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="F386" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="387">
@@ -30264,7 +30264,7 @@
         </is>
       </c>
       <c r="F463" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="464">
@@ -30354,7 +30354,7 @@
         </is>
       </c>
       <c r="F466" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="467">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>20.38</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-28 13:51:56 UTC</t>
+          <t>2026-08-29 08:42:15 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #31 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.158</v>
+        <v>0.261</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="F362" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G362" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.158</v>
+        <v>0.261</v>
       </c>
     </row>
     <row r="3">
@@ -17214,7 +17214,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="29">
@@ -17244,7 +17244,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="30">
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="36">
@@ -27234,7 +27234,7 @@
         </is>
       </c>
       <c r="F362" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="363">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.38</t>
+          <t>20.47</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-29 08:42:15 UTC</t>
+          <t>2026-08-30 07:57:25 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #32 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.261</v>
+        <v>0.317</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.261</v>
+        <v>0.317</v>
       </c>
     </row>
     <row r="3">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.47</t>
+          <t>20.55</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-30 07:57:25 UTC</t>
+          <t>2026-08-31 08:11:45 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #33 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.317</v>
+        <v>0.094</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.317</v>
+        <v>0.094</v>
       </c>
     </row>
     <row r="3">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="35">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.55</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-31 08:11:45 UTC</t>
+          <t>2026-09-01 07:21:29 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #34 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.094</v>
+        <v>0.23</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -12350,7 +12350,7 @@
         </is>
       </c>
       <c r="F382" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G382" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.094</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="3">
@@ -17394,7 +17394,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="35">
@@ -27834,7 +27834,7 @@
         </is>
       </c>
       <c r="F382" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="383">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>20.45</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-01 07:21:29 UTC</t>
+          <t>2026-09-02 06:53:35 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #35 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.23</v>
+        <v>0.096</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="F243" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G243" s="2" t="inlineStr"/>
     </row>
@@ -12350,7 +12350,7 @@
         </is>
       </c>
       <c r="F382" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G382" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.23</v>
+        <v>0.096</v>
       </c>
     </row>
     <row r="3">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="164">
@@ -23664,7 +23664,7 @@
         </is>
       </c>
       <c r="F243" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="244">
@@ -27834,7 +27834,7 @@
         </is>
       </c>
       <c r="F382" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="383">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.45</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-02 06:53:35 UTC</t>
+          <t>2026-09-03 06:56:05 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #36 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="G163" s="2" t="inlineStr"/>
     </row>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="F243" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="G243" s="2" t="inlineStr"/>
     </row>
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="20">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -21264,7 +21264,7 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="164">
@@ -23664,7 +23664,7 @@
         </is>
       </c>
       <c r="F243" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="244">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>20.30</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03 06:56:05 UTC</t>
+          <t>2026-09-04 07:00:52 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
deploy: Appium E2E Report – Build #37 (30ec4bcdc27ab8632665be11b7a484bbfceb8c5c) 30ec4bcdc27ab8632665be11b7a484bbfceb8c5c
</commit_message>
<xml_diff>
--- a/reports/latest/Reports/Automation_Test_Report.xlsx
+++ b/reports/latest/Reports/Automation_Test_Report.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.096</v>
+        <v>0.192</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
     </row>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
     </row>
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
     </row>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
     </row>
@@ -16434,7 +16434,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.096</v>
+        <v>0.192</v>
       </c>
     </row>
     <row r="3">
@@ -16944,7 +16944,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="20">
@@ -17724,7 +17724,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="46">
@@ -19164,7 +19164,7 @@
         </is>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="94">
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="95">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="97">
@@ -20724,7 +20724,7 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="146">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20.30</t>
+          <t>20.40</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -32002,7 +32002,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04 07:00:52 UTC</t>
+          <t>2026-09-05 06:45:26 UTC</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">

</xml_diff>